<commit_message>
change to crop value and add pkg titles
</commit_message>
<xml_diff>
--- a/data/raw/Example questionnaire.xlsx
+++ b/data/raw/Example questionnaire.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\au757887\PC_documents\_git-it\PPATonline\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDBFAA7F-DEEF-48C4-A47F-9E98BC6AA015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC9EFA9C-828B-4E90-8505-6F4B99584761}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DCB68ECE-DBFD-4EA5-81CC-7203B783D8F9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DCB68ECE-DBFD-4EA5-81CC-7203B783D8F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Example questionnaire" sheetId="1" r:id="rId1"/>
@@ -73,9 +73,6 @@
     <t>Time/management</t>
   </si>
   <si>
-    <t>Crop losses</t>
-  </si>
-  <si>
     <t>Direct costs</t>
   </si>
   <si>
@@ -86,6 +83,9 @@
   </si>
   <si>
     <t>User health and safety</t>
+  </si>
+  <si>
+    <t>Crop value</t>
   </si>
 </sst>
 </file>
@@ -947,34 +947,34 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C23ED5A6-8E82-40C8-856E-7E2516780679}">
   <dimension ref="A1:E18"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="3" width="22.6640625" customWidth="1"/>
-    <col min="4" max="4" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="22.7109375" customWidth="1"/>
+    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -991,12 +991,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C7">
         <v>50</v>
@@ -1008,9 +1008,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C8" t="s">
         <v>14</v>
@@ -1022,7 +1022,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>16</v>
       </c>
@@ -1036,9 +1036,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C10" t="s">
         <v>15</v>
@@ -1050,9 +1050,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C11" t="s">
         <v>14</v>
@@ -1064,9 +1064,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C12" t="s">
         <v>14</v>
@@ -1078,12 +1078,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C13">
         <v>50</v>
@@ -1095,9 +1095,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C14" t="s">
         <v>14</v>
@@ -1109,7 +1109,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>16</v>
       </c>
@@ -1123,9 +1123,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C16" t="s">
         <v>15</v>
@@ -1137,9 +1137,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C17" t="s">
         <v>14</v>
@@ -1151,9 +1151,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C18" t="s">
         <v>14</v>

</xml_diff>

<commit_message>
change titles of example questionaire
</commit_message>
<xml_diff>
--- a/data/raw/Example questionnaire.xlsx
+++ b/data/raw/Example questionnaire.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\au757887\PC_documents\_git-it\PPATonline\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2999976C-BB34-4452-90E9-42E68271F341}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB26B038-F25C-4620-8B62-C59C4B1A1AED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DCB68ECE-DBFD-4EA5-81CC-7203B783D8F9}"/>
   </bookViews>
@@ -65,9 +65,6 @@
     <t>Baseline - fungicides</t>
   </si>
   <si>
-    <t>New approach - fairy dust</t>
-  </si>
-  <si>
     <t>weight</t>
   </si>
   <si>
@@ -96,6 +93,9 @@
   </si>
   <si>
     <t>h</t>
+  </si>
+  <si>
+    <t>A new approach - fairy dust</t>
   </si>
 </sst>
 </file>
@@ -992,7 +992,7 @@
         <v>7</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D6" t="s">
         <v>1</v>
@@ -1006,7 +1006,7 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C7">
         <v>50</v>
@@ -1020,52 +1020,52 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D8">
         <v>3</v>
       </c>
       <c r="E8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D9">
         <v>3</v>
       </c>
       <c r="E9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D10">
         <v>3</v>
       </c>
       <c r="E10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D11">
         <v>4</v>
@@ -1076,24 +1076,24 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D12">
         <v>4</v>
       </c>
       <c r="E12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C13">
         <v>50</v>
@@ -1102,29 +1102,29 @@
         <v>5</v>
       </c>
       <c r="E13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C14" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D14">
         <v>3</v>
       </c>
       <c r="E14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D15">
         <v>4</v>
@@ -1135,24 +1135,24 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D16">
         <v>4</v>
       </c>
       <c r="E16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C17" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D17">
         <v>3</v>
@@ -1163,16 +1163,16 @@
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C18" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D18">
         <v>2</v>
       </c>
       <c r="E18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>